<commit_message>
Fix Excel spreadsheet downloads
</commit_message>
<xml_diff>
--- a/public/downloads/bill-payment-tracker.xlsx
+++ b/public/downloads/bill-payment-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="25">
   <si>
     <t>Bill Payment Tracker</t>
   </si>
@@ -177,15 +177,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -542,7 +545,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="22" customWidth="1"/>
@@ -584,7 +587,7 @@
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -604,185 +607,159 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>1200</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="4" t="s">
+      <c r="F4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="6">
         <v>110</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="4" t="s">
+      <c r="F5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="6">
         <v>45</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="F6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="6">
         <v>70</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="4" t="s">
+      <c r="F7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="6">
         <v>60</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="4" t="s">
+      <c r="F8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="7">
+      <c r="B9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="8">
         <f>SUM(C4:C8)</f>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" t="s">
-        <v>8</v>
-      </c>
-      <c r="H10" t="s">
-        <v>9</v>
+      <c r="D9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>